<commit_message>
feat(corpus): indexar catalogos Febi y TC-Matic + corpus combinado 283 entradas
Corpus AD Parts 115 entradas (fichas PDF), Febi 82, TC-Matic 72, equivalencias 14.
corpus_embeddings_completo.json: formato unificado {id, marca, triggerQuery, text}
Anade Productos TC-Matic Abril 2026.xlsx y Equivalencias Febi-TC-Matic.xlsx

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BASE DE CONOCIMIENTO/PRODUCTOS Y REFERENCIAS/Productos Febi Abril 2026.xlsx
+++ b/BASE DE CONOCIMIENTO/PRODUCTOS Y REFERENCIAS/Productos Febi Abril 2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RIB\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RIB\Documents\DOCUMENTOS RIB\DOCUMENTOS\CLAUDE\Proyectos\Buscador Aceites\BASE DE CONOCIMIENTO\PRODUCTOS Y REFERENCIAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608DBAE9-80EA-44C5-BA4B-EBD73C483E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460881A0-63BD-49BC-8AF9-C886B7CF9E8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2312" uniqueCount="543">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2322" uniqueCount="545">
   <si>
     <t>Marca</t>
   </si>
@@ -1164,9 +1164,6 @@
     <t>83 22 2 365 987</t>
   </si>
   <si>
-    <t>for direct shift gearbox (DCTF-1)</t>
-  </si>
-  <si>
     <t>G 052 529 A2</t>
   </si>
   <si>
@@ -1197,9 +1194,6 @@
     <t>75W-80</t>
   </si>
   <si>
-    <t>for direct shift gearbox (DCTF-2)</t>
-  </si>
-  <si>
     <t>G 055 529 A2</t>
   </si>
   <si>
@@ -1257,9 +1251,6 @@
     <t>02200-00110</t>
   </si>
   <si>
-    <t>for direct shift gearbox (DCTF-G)</t>
-  </si>
-  <si>
     <t>83 22 2 433 157</t>
   </si>
   <si>
@@ -1326,9 +1317,6 @@
     <t>Hydraulic Fluid</t>
   </si>
   <si>
-    <t>for hydropneumatic suspension and level control systems</t>
-  </si>
-  <si>
     <t>ACEITE PARA HIDRAULICA 1L</t>
   </si>
   <si>
@@ -1347,9 +1335,6 @@
     <t>06161</t>
   </si>
   <si>
-    <t>for central, power steering and level control systems</t>
-  </si>
-  <si>
     <t>83 29 0 429 576</t>
   </si>
   <si>
@@ -1359,15 +1344,9 @@
     <t>06162</t>
   </si>
   <si>
-    <t>for central hydraulic system</t>
-  </si>
-  <si>
     <t>81 22 9 407 549</t>
   </si>
   <si>
-    <t>for power steering system</t>
-  </si>
-  <si>
     <t>001 989 24 03</t>
   </si>
   <si>
@@ -1386,9 +1365,6 @@
     <t>Oil</t>
   </si>
   <si>
-    <t>for Haldex coupling</t>
-  </si>
-  <si>
     <t>ACEITE PARA EMBRAGUE HALDEX</t>
   </si>
   <si>
@@ -1428,9 +1404,6 @@
     <t>Transfer Case Fluid</t>
   </si>
   <si>
-    <t>TF-1</t>
-  </si>
-  <si>
     <t>83 22 2 409 710</t>
   </si>
   <si>
@@ -1657,6 +1630,39 @@
   </si>
   <si>
     <t>BMW - DTF-1; MB - 239.41; TF 0870; TF0870B.</t>
+  </si>
+  <si>
+    <t>Embrague Haldex</t>
+  </si>
+  <si>
+    <t>Caja de Transferencia TF-1</t>
+  </si>
+  <si>
+    <t>Servodirección</t>
+  </si>
+  <si>
+    <t>1003306</t>
+  </si>
+  <si>
+    <t>Servodireccion e Hidráulica</t>
+  </si>
+  <si>
+    <t>Cambio marchas directo (DCTF-1)</t>
+  </si>
+  <si>
+    <t>Cambio marchas directo (DCTF-2)</t>
+  </si>
+  <si>
+    <t>Cambio marchas directo (DCTF-G)</t>
+  </si>
+  <si>
+    <t>Suspension Hydroneumática y Regulación Nivel</t>
+  </si>
+  <si>
+    <t>Hidraulica Central , Sevodireccion y Control de Nivel</t>
+  </si>
+  <si>
+    <t>Hidráulica Central</t>
   </si>
 </sst>
 </file>
@@ -1780,7 +1786,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1819,11 +1825,23 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -2256,7 +2274,7 @@
       <c r="T2" s="2"/>
       <c r="U2" s="2"/>
       <c r="V2" s="2" t="s">
-        <v>474</v>
+        <v>465</v>
       </c>
     </row>
     <row r="3" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2298,7 +2316,7 @@
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
       <c r="V3" s="2" t="s">
-        <v>474</v>
+        <v>465</v>
       </c>
     </row>
     <row r="4" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2340,7 +2358,7 @@
       <c r="T4" s="2"/>
       <c r="U4" s="2"/>
       <c r="V4" s="2" t="s">
-        <v>474</v>
+        <v>465</v>
       </c>
     </row>
     <row r="5" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2382,7 +2400,7 @@
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
       <c r="V5" s="2" t="s">
-        <v>474</v>
+        <v>465</v>
       </c>
     </row>
     <row r="6" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2424,7 +2442,7 @@
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
       <c r="V6" s="2" t="s">
-        <v>474</v>
+        <v>465</v>
       </c>
     </row>
     <row r="7" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2466,7 +2484,7 @@
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
       <c r="V7" s="2" t="s">
-        <v>474</v>
+        <v>465</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2512,7 +2530,7 @@
         <v>33</v>
       </c>
       <c r="V8" s="2" t="s">
-        <v>475</v>
+        <v>466</v>
       </c>
     </row>
     <row r="9" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2558,7 +2576,7 @@
         <v>33</v>
       </c>
       <c r="V9" s="2" t="s">
-        <v>475</v>
+        <v>466</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2604,7 +2622,7 @@
         <v>33</v>
       </c>
       <c r="V10" s="2" t="s">
-        <v>475</v>
+        <v>466</v>
       </c>
     </row>
     <row r="11" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2648,7 +2666,7 @@
         <v>39</v>
       </c>
       <c r="V11" s="2" t="s">
-        <v>476</v>
+        <v>467</v>
       </c>
     </row>
     <row r="12" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2692,7 +2710,7 @@
         <v>39</v>
       </c>
       <c r="V12" s="2" t="s">
-        <v>476</v>
+        <v>467</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2736,7 +2754,7 @@
         <v>39</v>
       </c>
       <c r="V13" s="2" t="s">
-        <v>476</v>
+        <v>467</v>
       </c>
     </row>
     <row r="14" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2782,7 +2800,7 @@
         <v>42</v>
       </c>
       <c r="V14" s="2" t="s">
-        <v>477</v>
+        <v>468</v>
       </c>
     </row>
     <row r="15" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2828,7 +2846,7 @@
         <v>42</v>
       </c>
       <c r="V15" s="2" t="s">
-        <v>477</v>
+        <v>468</v>
       </c>
     </row>
     <row r="16" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2874,7 +2892,7 @@
         <v>42</v>
       </c>
       <c r="V16" s="2" t="s">
-        <v>477</v>
+        <v>468</v>
       </c>
     </row>
     <row r="17" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2920,7 +2938,7 @@
         <v>42</v>
       </c>
       <c r="V17" s="2" t="s">
-        <v>477</v>
+        <v>468</v>
       </c>
     </row>
     <row r="18" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -2966,7 +2984,7 @@
         <v>42</v>
       </c>
       <c r="V18" s="2" t="s">
-        <v>477</v>
+        <v>468</v>
       </c>
     </row>
     <row r="19" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3010,7 +3028,7 @@
       <c r="T19" s="2"/>
       <c r="U19" s="2"/>
       <c r="V19" s="2" t="s">
-        <v>478</v>
+        <v>469</v>
       </c>
     </row>
     <row r="20" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3054,7 +3072,7 @@
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
       <c r="V20" s="2" t="s">
-        <v>478</v>
+        <v>469</v>
       </c>
     </row>
     <row r="21" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3100,7 +3118,7 @@
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
       <c r="V21" s="2" t="s">
-        <v>478</v>
+        <v>469</v>
       </c>
     </row>
     <row r="22" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3146,7 +3164,7 @@
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
       <c r="V22" s="2" t="s">
-        <v>478</v>
+        <v>469</v>
       </c>
     </row>
     <row r="23" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3190,7 +3208,7 @@
         <v>57</v>
       </c>
       <c r="V23" s="2" t="s">
-        <v>479</v>
+        <v>470</v>
       </c>
     </row>
     <row r="24" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3234,7 +3252,7 @@
         <v>57</v>
       </c>
       <c r="V24" s="2" t="s">
-        <v>479</v>
+        <v>470</v>
       </c>
     </row>
     <row r="25" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3278,7 +3296,7 @@
         <v>57</v>
       </c>
       <c r="V25" s="2" t="s">
-        <v>479</v>
+        <v>470</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3322,7 +3340,7 @@
         <v>57</v>
       </c>
       <c r="V26" s="2" t="s">
-        <v>479</v>
+        <v>470</v>
       </c>
     </row>
     <row r="27" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3366,7 +3384,7 @@
         <v>60</v>
       </c>
       <c r="V27" s="2" t="s">
-        <v>480</v>
+        <v>471</v>
       </c>
     </row>
     <row r="28" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3410,7 +3428,7 @@
         <v>60</v>
       </c>
       <c r="V28" s="2" t="s">
-        <v>480</v>
+        <v>471</v>
       </c>
     </row>
     <row r="29" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3454,7 +3472,7 @@
         <v>60</v>
       </c>
       <c r="V29" s="2" t="s">
-        <v>480</v>
+        <v>471</v>
       </c>
     </row>
     <row r="30" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3498,7 +3516,7 @@
         <v>60</v>
       </c>
       <c r="V30" s="2" t="s">
-        <v>480</v>
+        <v>471</v>
       </c>
     </row>
     <row r="31" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3542,7 +3560,7 @@
         <v>60</v>
       </c>
       <c r="V31" s="2" t="s">
-        <v>480</v>
+        <v>471</v>
       </c>
     </row>
     <row r="32" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3586,7 +3604,7 @@
         <v>67</v>
       </c>
       <c r="V32" s="2" t="s">
-        <v>481</v>
+        <v>472</v>
       </c>
     </row>
     <row r="33" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3630,7 +3648,7 @@
         <v>67</v>
       </c>
       <c r="V33" s="2" t="s">
-        <v>481</v>
+        <v>472</v>
       </c>
     </row>
     <row r="34" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3674,7 +3692,7 @@
         <v>67</v>
       </c>
       <c r="V34" s="2" t="s">
-        <v>481</v>
+        <v>472</v>
       </c>
     </row>
     <row r="35" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3718,7 +3736,7 @@
         <v>67</v>
       </c>
       <c r="V35" s="2" t="s">
-        <v>481</v>
+        <v>472</v>
       </c>
     </row>
     <row r="36" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3762,7 +3780,7 @@
         <v>67</v>
       </c>
       <c r="V36" s="2" t="s">
-        <v>481</v>
+        <v>472</v>
       </c>
     </row>
     <row r="37" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3806,7 +3824,7 @@
         <v>73</v>
       </c>
       <c r="V37" s="2" t="s">
-        <v>482</v>
+        <v>473</v>
       </c>
     </row>
     <row r="38" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3850,7 +3868,7 @@
         <v>73</v>
       </c>
       <c r="V38" s="2" t="s">
-        <v>482</v>
+        <v>473</v>
       </c>
     </row>
     <row r="39" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3894,7 +3912,7 @@
         <v>73</v>
       </c>
       <c r="V39" s="2" t="s">
-        <v>482</v>
+        <v>473</v>
       </c>
     </row>
     <row r="40" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3938,7 +3956,7 @@
         <v>73</v>
       </c>
       <c r="V40" s="2" t="s">
-        <v>482</v>
+        <v>473</v>
       </c>
     </row>
     <row r="41" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -3982,7 +4000,7 @@
         <v>73</v>
       </c>
       <c r="V41" s="2" t="s">
-        <v>482</v>
+        <v>473</v>
       </c>
     </row>
     <row r="42" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4026,7 +4044,7 @@
         <v>77</v>
       </c>
       <c r="V42" s="2" t="s">
-        <v>483</v>
+        <v>474</v>
       </c>
     </row>
     <row r="43" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4070,7 +4088,7 @@
         <v>77</v>
       </c>
       <c r="V43" s="2" t="s">
-        <v>483</v>
+        <v>474</v>
       </c>
     </row>
     <row r="44" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4114,7 +4132,7 @@
         <v>77</v>
       </c>
       <c r="V44" s="2" t="s">
-        <v>483</v>
+        <v>474</v>
       </c>
     </row>
     <row r="45" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4158,7 +4176,7 @@
         <v>77</v>
       </c>
       <c r="V45" s="2" t="s">
-        <v>483</v>
+        <v>474</v>
       </c>
     </row>
     <row r="46" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4202,7 +4220,7 @@
         <v>77</v>
       </c>
       <c r="V46" s="2" t="s">
-        <v>483</v>
+        <v>474</v>
       </c>
     </row>
     <row r="47" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4246,7 +4264,7 @@
         <v>84</v>
       </c>
       <c r="V47" s="2" t="s">
-        <v>484</v>
+        <v>475</v>
       </c>
     </row>
     <row r="48" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4290,7 +4308,7 @@
         <v>84</v>
       </c>
       <c r="V48" s="2" t="s">
-        <v>484</v>
+        <v>475</v>
       </c>
     </row>
     <row r="49" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4334,7 +4352,7 @@
         <v>84</v>
       </c>
       <c r="V49" s="2" t="s">
-        <v>484</v>
+        <v>475</v>
       </c>
     </row>
     <row r="50" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4378,7 +4396,7 @@
         <v>84</v>
       </c>
       <c r="V50" s="2" t="s">
-        <v>484</v>
+        <v>475</v>
       </c>
     </row>
     <row r="51" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4422,7 +4440,7 @@
         <v>84</v>
       </c>
       <c r="V51" s="2" t="s">
-        <v>484</v>
+        <v>475</v>
       </c>
     </row>
     <row r="52" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4466,7 +4484,7 @@
         <v>90</v>
       </c>
       <c r="V52" s="2" t="s">
-        <v>485</v>
+        <v>476</v>
       </c>
     </row>
     <row r="53" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4510,7 +4528,7 @@
         <v>90</v>
       </c>
       <c r="V53" s="2" t="s">
-        <v>485</v>
+        <v>476</v>
       </c>
     </row>
     <row r="54" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4554,7 +4572,7 @@
         <v>90</v>
       </c>
       <c r="V54" s="2" t="s">
-        <v>485</v>
+        <v>476</v>
       </c>
     </row>
     <row r="55" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4598,7 +4616,7 @@
         <v>90</v>
       </c>
       <c r="V55" s="2" t="s">
-        <v>485</v>
+        <v>476</v>
       </c>
     </row>
     <row r="56" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4642,7 +4660,7 @@
         <v>90</v>
       </c>
       <c r="V56" s="2" t="s">
-        <v>485</v>
+        <v>476</v>
       </c>
     </row>
     <row r="57" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4818,7 +4836,7 @@
         <v>96</v>
       </c>
       <c r="V60" s="2" t="s">
-        <v>486</v>
+        <v>477</v>
       </c>
     </row>
     <row r="61" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4862,7 +4880,7 @@
         <v>96</v>
       </c>
       <c r="V61" s="2" t="s">
-        <v>486</v>
+        <v>477</v>
       </c>
     </row>
     <row r="62" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4906,7 +4924,7 @@
         <v>96</v>
       </c>
       <c r="V62" s="2" t="s">
-        <v>486</v>
+        <v>477</v>
       </c>
     </row>
     <row r="63" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -4956,7 +4974,7 @@
         <v>104</v>
       </c>
       <c r="V63" s="2" t="s">
-        <v>487</v>
+        <v>478</v>
       </c>
     </row>
     <row r="64" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5008,7 +5026,7 @@
         <v>104</v>
       </c>
       <c r="V64" s="2" t="s">
-        <v>487</v>
+        <v>478</v>
       </c>
     </row>
     <row r="65" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5058,7 +5076,7 @@
         <v>104</v>
       </c>
       <c r="V65" s="2" t="s">
-        <v>487</v>
+        <v>478</v>
       </c>
     </row>
     <row r="66" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5108,7 +5126,7 @@
         <v>104</v>
       </c>
       <c r="V66" s="2" t="s">
-        <v>487</v>
+        <v>478</v>
       </c>
     </row>
     <row r="67" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5156,7 +5174,7 @@
       <c r="T67" s="2"/>
       <c r="U67" s="2"/>
       <c r="V67" s="2" t="s">
-        <v>488</v>
+        <v>479</v>
       </c>
     </row>
     <row r="68" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5206,7 +5224,7 @@
       <c r="T68" s="2"/>
       <c r="U68" s="2"/>
       <c r="V68" s="2" t="s">
-        <v>488</v>
+        <v>479</v>
       </c>
     </row>
     <row r="69" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5254,7 +5272,7 @@
       <c r="T69" s="2"/>
       <c r="U69" s="2"/>
       <c r="V69" s="2" t="s">
-        <v>488</v>
+        <v>479</v>
       </c>
     </row>
     <row r="70" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5302,7 +5320,7 @@
       <c r="T70" s="2"/>
       <c r="U70" s="2"/>
       <c r="V70" s="2" t="s">
-        <v>488</v>
+        <v>479</v>
       </c>
     </row>
     <row r="71" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5350,7 +5368,7 @@
       <c r="T71" s="2"/>
       <c r="U71" s="2"/>
       <c r="V71" s="2" t="s">
-        <v>489</v>
+        <v>480</v>
       </c>
     </row>
     <row r="72" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5400,7 +5418,7 @@
       <c r="T72" s="2"/>
       <c r="U72" s="2"/>
       <c r="V72" s="2" t="s">
-        <v>489</v>
+        <v>480</v>
       </c>
     </row>
     <row r="73" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5448,7 +5466,7 @@
       <c r="T73" s="2"/>
       <c r="U73" s="2"/>
       <c r="V73" s="2" t="s">
-        <v>489</v>
+        <v>480</v>
       </c>
     </row>
     <row r="74" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5496,7 +5514,7 @@
       <c r="T74" s="2"/>
       <c r="U74" s="2"/>
       <c r="V74" s="2" t="s">
-        <v>489</v>
+        <v>480</v>
       </c>
     </row>
     <row r="75" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5548,7 +5566,7 @@
         <v>127</v>
       </c>
       <c r="V75" s="2" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
     </row>
     <row r="76" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5600,7 +5618,7 @@
         <v>127</v>
       </c>
       <c r="V76" s="2" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
     </row>
     <row r="77" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5652,7 +5670,7 @@
         <v>127</v>
       </c>
       <c r="V77" s="2" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
     </row>
     <row r="78" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5704,7 +5722,7 @@
         <v>135</v>
       </c>
       <c r="V78" s="2" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
     </row>
     <row r="79" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5756,7 +5774,7 @@
         <v>135</v>
       </c>
       <c r="V79" s="2" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
     </row>
     <row r="80" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5808,7 +5826,7 @@
         <v>135</v>
       </c>
       <c r="V80" s="2" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
     </row>
     <row r="81" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5860,7 +5878,7 @@
         <v>135</v>
       </c>
       <c r="V81" s="2" t="s">
-        <v>490</v>
+        <v>481</v>
       </c>
     </row>
     <row r="82" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -5998,7 +6016,7 @@
         <v>149</v>
       </c>
       <c r="V84" s="2" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
     </row>
     <row r="85" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6046,7 +6064,7 @@
         <v>149</v>
       </c>
       <c r="V85" s="2" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
     </row>
     <row r="86" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6094,7 +6112,7 @@
         <v>149</v>
       </c>
       <c r="V86" s="2" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
     </row>
     <row r="87" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6142,7 +6160,7 @@
         <v>149</v>
       </c>
       <c r="V87" s="2" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
     </row>
     <row r="88" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6190,7 +6208,7 @@
         <v>149</v>
       </c>
       <c r="V88" s="2" t="s">
-        <v>491</v>
+        <v>482</v>
       </c>
     </row>
     <row r="89" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6480,7 +6498,7 @@
         <v>173</v>
       </c>
       <c r="V94" s="2" t="s">
-        <v>492</v>
+        <v>483</v>
       </c>
     </row>
     <row r="95" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6528,7 +6546,7 @@
         <v>173</v>
       </c>
       <c r="V95" s="2" t="s">
-        <v>492</v>
+        <v>483</v>
       </c>
     </row>
     <row r="96" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6576,7 +6594,7 @@
         <v>173</v>
       </c>
       <c r="V96" s="2" t="s">
-        <v>492</v>
+        <v>483</v>
       </c>
     </row>
     <row r="97" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6624,7 +6642,7 @@
         <v>173</v>
       </c>
       <c r="V97" s="2" t="s">
-        <v>492</v>
+        <v>483</v>
       </c>
     </row>
     <row r="98" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6672,7 +6690,7 @@
         <v>173</v>
       </c>
       <c r="V98" s="2" t="s">
-        <v>492</v>
+        <v>483</v>
       </c>
     </row>
     <row r="99" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6872,7 +6890,7 @@
         <v>186</v>
       </c>
       <c r="V102" s="2" t="s">
-        <v>493</v>
+        <v>484</v>
       </c>
     </row>
     <row r="103" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6922,7 +6940,7 @@
         <v>186</v>
       </c>
       <c r="V103" s="2" t="s">
-        <v>493</v>
+        <v>484</v>
       </c>
     </row>
     <row r="104" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -6972,7 +6990,7 @@
         <v>186</v>
       </c>
       <c r="V104" s="2" t="s">
-        <v>493</v>
+        <v>484</v>
       </c>
     </row>
     <row r="105" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7068,7 +7086,7 @@
         <v>196</v>
       </c>
       <c r="V106" s="2" t="s">
-        <v>494</v>
+        <v>485</v>
       </c>
     </row>
     <row r="107" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7116,7 +7134,7 @@
         <v>196</v>
       </c>
       <c r="V107" s="2" t="s">
-        <v>494</v>
+        <v>485</v>
       </c>
     </row>
     <row r="108" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7164,7 +7182,7 @@
         <v>196</v>
       </c>
       <c r="V108" s="2" t="s">
-        <v>494</v>
+        <v>485</v>
       </c>
     </row>
     <row r="109" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7212,7 +7230,7 @@
         <v>201</v>
       </c>
       <c r="V109" s="2" t="s">
-        <v>495</v>
+        <v>486</v>
       </c>
     </row>
     <row r="110" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7260,7 +7278,7 @@
         <v>201</v>
       </c>
       <c r="V110" s="2" t="s">
-        <v>495</v>
+        <v>486</v>
       </c>
     </row>
     <row r="111" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7308,7 +7326,7 @@
         <v>201</v>
       </c>
       <c r="V111" s="2" t="s">
-        <v>495</v>
+        <v>486</v>
       </c>
     </row>
     <row r="112" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7358,7 +7376,7 @@
         <v>206</v>
       </c>
       <c r="V112" s="2" t="s">
-        <v>496</v>
+        <v>487</v>
       </c>
     </row>
     <row r="113" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7408,7 +7426,7 @@
         <v>206</v>
       </c>
       <c r="V113" s="2" t="s">
-        <v>496</v>
+        <v>487</v>
       </c>
     </row>
     <row r="114" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7458,7 +7476,7 @@
         <v>206</v>
       </c>
       <c r="V114" s="2" t="s">
-        <v>496</v>
+        <v>487</v>
       </c>
     </row>
     <row r="115" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7508,7 +7526,7 @@
         <v>208</v>
       </c>
       <c r="V115" s="2" t="s">
-        <v>497</v>
+        <v>488</v>
       </c>
     </row>
     <row r="116" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7558,7 +7576,7 @@
         <v>208</v>
       </c>
       <c r="V116" s="2" t="s">
-        <v>497</v>
+        <v>488</v>
       </c>
     </row>
     <row r="117" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7608,7 +7626,7 @@
         <v>208</v>
       </c>
       <c r="V117" s="2" t="s">
-        <v>497</v>
+        <v>488</v>
       </c>
     </row>
     <row r="118" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7658,7 +7676,7 @@
         <v>211</v>
       </c>
       <c r="V118" s="2" t="s">
-        <v>498</v>
+        <v>489</v>
       </c>
     </row>
     <row r="119" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7708,7 +7726,7 @@
         <v>211</v>
       </c>
       <c r="V119" s="2" t="s">
-        <v>498</v>
+        <v>489</v>
       </c>
     </row>
     <row r="120" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7758,7 +7776,7 @@
         <v>211</v>
       </c>
       <c r="V120" s="2" t="s">
-        <v>498</v>
+        <v>489</v>
       </c>
     </row>
     <row r="121" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7808,7 +7826,7 @@
         <v>213</v>
       </c>
       <c r="V121" s="2" t="s">
-        <v>499</v>
+        <v>490</v>
       </c>
     </row>
     <row r="122" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7858,7 +7876,7 @@
         <v>213</v>
       </c>
       <c r="V122" s="2" t="s">
-        <v>499</v>
+        <v>490</v>
       </c>
     </row>
     <row r="123" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7908,7 +7926,7 @@
         <v>213</v>
       </c>
       <c r="V123" s="2" t="s">
-        <v>499</v>
+        <v>490</v>
       </c>
     </row>
     <row r="124" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7958,7 +7976,7 @@
         <v>218</v>
       </c>
       <c r="V124" s="2" t="s">
-        <v>500</v>
+        <v>491</v>
       </c>
     </row>
     <row r="125" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8008,7 +8026,7 @@
         <v>218</v>
       </c>
       <c r="V125" s="2" t="s">
-        <v>500</v>
+        <v>491</v>
       </c>
     </row>
     <row r="126" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8058,7 +8076,7 @@
         <v>218</v>
       </c>
       <c r="V126" s="2" t="s">
-        <v>500</v>
+        <v>491</v>
       </c>
     </row>
     <row r="127" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8108,7 +8126,7 @@
         <v>223</v>
       </c>
       <c r="V127" s="2" t="s">
-        <v>501</v>
+        <v>492</v>
       </c>
     </row>
     <row r="128" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8158,7 +8176,7 @@
         <v>223</v>
       </c>
       <c r="V128" s="2" t="s">
-        <v>501</v>
+        <v>492</v>
       </c>
     </row>
     <row r="129" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8208,7 +8226,7 @@
         <v>223</v>
       </c>
       <c r="V129" s="2" t="s">
-        <v>501</v>
+        <v>492</v>
       </c>
     </row>
     <row r="130" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8258,7 +8276,7 @@
         <v>231</v>
       </c>
       <c r="V130" s="2" t="s">
-        <v>502</v>
+        <v>493</v>
       </c>
     </row>
     <row r="131" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8308,7 +8326,7 @@
         <v>231</v>
       </c>
       <c r="V131" s="2" t="s">
-        <v>502</v>
+        <v>493</v>
       </c>
     </row>
     <row r="132" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8358,7 +8376,7 @@
         <v>231</v>
       </c>
       <c r="V132" s="2" t="s">
-        <v>502</v>
+        <v>493</v>
       </c>
     </row>
     <row r="133" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8408,7 +8426,7 @@
         <v>231</v>
       </c>
       <c r="V133" s="2" t="s">
-        <v>502</v>
+        <v>493</v>
       </c>
     </row>
     <row r="134" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8458,7 +8476,7 @@
         <v>231</v>
       </c>
       <c r="V134" s="2" t="s">
-        <v>502</v>
+        <v>493</v>
       </c>
     </row>
     <row r="135" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8508,7 +8526,7 @@
         <v>245</v>
       </c>
       <c r="V135" s="2" t="s">
-        <v>503</v>
+        <v>494</v>
       </c>
     </row>
     <row r="136" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8558,7 +8576,7 @@
         <v>245</v>
       </c>
       <c r="V136" s="2" t="s">
-        <v>503</v>
+        <v>494</v>
       </c>
     </row>
     <row r="137" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8610,7 +8628,7 @@
         <v>245</v>
       </c>
       <c r="V137" s="2" t="s">
-        <v>503</v>
+        <v>494</v>
       </c>
     </row>
     <row r="138" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8660,7 +8678,7 @@
         <v>245</v>
       </c>
       <c r="V138" s="2" t="s">
-        <v>503</v>
+        <v>494</v>
       </c>
     </row>
     <row r="139" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8710,7 +8728,7 @@
         <v>245</v>
       </c>
       <c r="V139" s="2" t="s">
-        <v>503</v>
+        <v>494</v>
       </c>
     </row>
     <row r="140" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8760,7 +8778,7 @@
         <v>245</v>
       </c>
       <c r="V140" s="2" t="s">
-        <v>503</v>
+        <v>494</v>
       </c>
     </row>
     <row r="141" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8810,7 +8828,7 @@
         <v>256</v>
       </c>
       <c r="V141" s="2" t="s">
-        <v>504</v>
+        <v>495</v>
       </c>
     </row>
     <row r="142" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8860,7 +8878,7 @@
         <v>256</v>
       </c>
       <c r="V142" s="2" t="s">
-        <v>504</v>
+        <v>495</v>
       </c>
     </row>
     <row r="143" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8910,7 +8928,7 @@
         <v>256</v>
       </c>
       <c r="V143" s="2" t="s">
-        <v>504</v>
+        <v>495</v>
       </c>
     </row>
     <row r="144" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -8960,7 +8978,7 @@
         <v>256</v>
       </c>
       <c r="V144" s="2" t="s">
-        <v>504</v>
+        <v>495</v>
       </c>
     </row>
     <row r="145" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9010,7 +9028,7 @@
         <v>256</v>
       </c>
       <c r="V145" s="2" t="s">
-        <v>504</v>
+        <v>495</v>
       </c>
     </row>
     <row r="146" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9060,7 +9078,7 @@
         <v>265</v>
       </c>
       <c r="V146" s="2" t="s">
-        <v>505</v>
+        <v>496</v>
       </c>
     </row>
     <row r="147" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9110,7 +9128,7 @@
         <v>265</v>
       </c>
       <c r="V147" s="2" t="s">
-        <v>505</v>
+        <v>496</v>
       </c>
     </row>
     <row r="148" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9160,7 +9178,7 @@
         <v>265</v>
       </c>
       <c r="V148" s="2" t="s">
-        <v>505</v>
+        <v>496</v>
       </c>
     </row>
     <row r="149" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9210,7 +9228,7 @@
         <v>265</v>
       </c>
       <c r="V149" s="2" t="s">
-        <v>505</v>
+        <v>496</v>
       </c>
     </row>
     <row r="150" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9260,7 +9278,7 @@
         <v>265</v>
       </c>
       <c r="V150" s="2" t="s">
-        <v>505</v>
+        <v>496</v>
       </c>
     </row>
     <row r="151" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9310,7 +9328,7 @@
         <v>274</v>
       </c>
       <c r="V151" s="2" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
     </row>
     <row r="152" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9360,7 +9378,7 @@
         <v>274</v>
       </c>
       <c r="V152" s="2" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
     </row>
     <row r="153" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9410,7 +9428,7 @@
         <v>274</v>
       </c>
       <c r="V153" s="2" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
     </row>
     <row r="154" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9462,7 +9480,7 @@
         <v>274</v>
       </c>
       <c r="V154" s="2" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
     </row>
     <row r="155" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9512,7 +9530,7 @@
         <v>274</v>
       </c>
       <c r="V155" s="2" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
     </row>
     <row r="156" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9562,7 +9580,7 @@
         <v>274</v>
       </c>
       <c r="V156" s="2" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
     </row>
     <row r="157" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9612,7 +9630,7 @@
         <v>274</v>
       </c>
       <c r="V157" s="2" t="s">
-        <v>506</v>
+        <v>497</v>
       </c>
     </row>
     <row r="158" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9662,7 +9680,7 @@
         <v>283</v>
       </c>
       <c r="V158" s="2" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
     </row>
     <row r="159" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9712,7 +9730,7 @@
         <v>283</v>
       </c>
       <c r="V159" s="2" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
     </row>
     <row r="160" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9762,7 +9780,7 @@
         <v>283</v>
       </c>
       <c r="V160" s="2" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
     </row>
     <row r="161" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9812,7 +9830,7 @@
         <v>283</v>
       </c>
       <c r="V161" s="2" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
     </row>
     <row r="162" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9862,7 +9880,7 @@
         <v>283</v>
       </c>
       <c r="V162" s="2" t="s">
-        <v>507</v>
+        <v>498</v>
       </c>
     </row>
     <row r="163" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9914,7 +9932,7 @@
         <v>293</v>
       </c>
       <c r="V163" s="2" t="s">
-        <v>508</v>
+        <v>499</v>
       </c>
     </row>
     <row r="164" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -9966,7 +9984,7 @@
         <v>293</v>
       </c>
       <c r="V164" s="2" t="s">
-        <v>508</v>
+        <v>499</v>
       </c>
     </row>
     <row r="165" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10018,7 +10036,7 @@
         <v>293</v>
       </c>
       <c r="V165" s="2" t="s">
-        <v>508</v>
+        <v>499</v>
       </c>
     </row>
     <row r="166" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10068,7 +10086,7 @@
         <v>297</v>
       </c>
       <c r="V166" s="2" t="s">
-        <v>509</v>
+        <v>500</v>
       </c>
     </row>
     <row r="167" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10118,7 +10136,7 @@
         <v>297</v>
       </c>
       <c r="V167" s="2" t="s">
-        <v>509</v>
+        <v>500</v>
       </c>
     </row>
     <row r="168" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10168,7 +10186,7 @@
         <v>297</v>
       </c>
       <c r="V168" s="2" t="s">
-        <v>509</v>
+        <v>500</v>
       </c>
     </row>
     <row r="169" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10218,7 +10236,7 @@
         <v>297</v>
       </c>
       <c r="V169" s="2" t="s">
-        <v>509</v>
+        <v>500</v>
       </c>
     </row>
     <row r="170" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10270,7 +10288,7 @@
         <v>306</v>
       </c>
       <c r="V170" s="2" t="s">
-        <v>510</v>
+        <v>501</v>
       </c>
     </row>
     <row r="171" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10322,7 +10340,7 @@
         <v>306</v>
       </c>
       <c r="V171" s="2" t="s">
-        <v>510</v>
+        <v>501</v>
       </c>
     </row>
     <row r="172" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10374,7 +10392,7 @@
         <v>306</v>
       </c>
       <c r="V172" s="2" t="s">
-        <v>510</v>
+        <v>501</v>
       </c>
     </row>
     <row r="173" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10426,7 +10444,7 @@
         <v>306</v>
       </c>
       <c r="V173" s="2" t="s">
-        <v>510</v>
+        <v>501</v>
       </c>
     </row>
     <row r="174" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10478,7 +10496,7 @@
         <v>312</v>
       </c>
       <c r="V174" s="2" t="s">
-        <v>511</v>
+        <v>502</v>
       </c>
     </row>
     <row r="175" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10530,7 +10548,7 @@
         <v>312</v>
       </c>
       <c r="V175" s="2" t="s">
-        <v>511</v>
+        <v>502</v>
       </c>
     </row>
     <row r="176" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10582,7 +10600,7 @@
         <v>318</v>
       </c>
       <c r="V176" s="2" t="s">
-        <v>512</v>
+        <v>503</v>
       </c>
     </row>
     <row r="177" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10634,7 +10652,7 @@
         <v>318</v>
       </c>
       <c r="V177" s="2" t="s">
-        <v>512</v>
+        <v>503</v>
       </c>
     </row>
     <row r="178" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10686,7 +10704,7 @@
         <v>318</v>
       </c>
       <c r="V178" s="2" t="s">
-        <v>512</v>
+        <v>503</v>
       </c>
     </row>
     <row r="179" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10734,7 +10752,7 @@
         <v>322</v>
       </c>
       <c r="V179" s="2" t="s">
-        <v>513</v>
+        <v>504</v>
       </c>
     </row>
     <row r="180" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10782,7 +10800,7 @@
         <v>322</v>
       </c>
       <c r="V180" s="2" t="s">
-        <v>513</v>
+        <v>504</v>
       </c>
     </row>
     <row r="181" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10830,7 +10848,7 @@
         <v>322</v>
       </c>
       <c r="V181" s="2" t="s">
-        <v>513</v>
+        <v>504</v>
       </c>
     </row>
     <row r="182" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10880,7 +10898,7 @@
         <v>327</v>
       </c>
       <c r="V182" s="2" t="s">
-        <v>514</v>
+        <v>505</v>
       </c>
     </row>
     <row r="183" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10930,7 +10948,7 @@
         <v>333</v>
       </c>
       <c r="V183" s="2" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
     </row>
     <row r="184" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -10980,7 +10998,7 @@
         <v>333</v>
       </c>
       <c r="V184" s="2" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
     </row>
     <row r="185" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11032,7 +11050,7 @@
         <v>333</v>
       </c>
       <c r="V185" s="2" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
     </row>
     <row r="186" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11080,7 +11098,7 @@
         <v>336</v>
       </c>
       <c r="V186" s="2" t="s">
-        <v>516</v>
+        <v>507</v>
       </c>
     </row>
     <row r="187" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11128,7 +11146,7 @@
         <v>336</v>
       </c>
       <c r="V187" s="2" t="s">
-        <v>516</v>
+        <v>507</v>
       </c>
     </row>
     <row r="188" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11176,7 +11194,7 @@
         <v>336</v>
       </c>
       <c r="V188" s="2" t="s">
-        <v>516</v>
+        <v>507</v>
       </c>
     </row>
     <row r="189" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11226,7 +11244,7 @@
         <v>340</v>
       </c>
       <c r="V189" s="2" t="s">
-        <v>517</v>
+        <v>508</v>
       </c>
     </row>
     <row r="190" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11276,7 +11294,7 @@
         <v>340</v>
       </c>
       <c r="V190" s="2" t="s">
-        <v>517</v>
+        <v>508</v>
       </c>
     </row>
     <row r="191" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11326,7 +11344,7 @@
         <v>340</v>
       </c>
       <c r="V191" s="2" t="s">
-        <v>517</v>
+        <v>508</v>
       </c>
     </row>
     <row r="192" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11382,7 +11400,7 @@
         <v>349</v>
       </c>
       <c r="V192" s="2" t="s">
-        <v>518</v>
+        <v>509</v>
       </c>
     </row>
     <row r="193" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11438,7 +11456,7 @@
         <v>349</v>
       </c>
       <c r="V193" s="2" t="s">
-        <v>518</v>
+        <v>509</v>
       </c>
     </row>
     <row r="194" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11494,7 +11512,7 @@
         <v>349</v>
       </c>
       <c r="V194" s="2" t="s">
-        <v>518</v>
+        <v>509</v>
       </c>
     </row>
     <row r="195" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11546,7 +11564,7 @@
         <v>353</v>
       </c>
       <c r="V195" s="2" t="s">
-        <v>519</v>
+        <v>510</v>
       </c>
     </row>
     <row r="196" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11598,7 +11616,7 @@
         <v>353</v>
       </c>
       <c r="V196" s="2" t="s">
-        <v>519</v>
+        <v>510</v>
       </c>
     </row>
     <row r="197" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11650,7 +11668,7 @@
         <v>353</v>
       </c>
       <c r="V197" s="2" t="s">
-        <v>519</v>
+        <v>510</v>
       </c>
     </row>
     <row r="198" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11702,7 +11720,7 @@
         <v>353</v>
       </c>
       <c r="V198" s="2" t="s">
-        <v>519</v>
+        <v>510</v>
       </c>
     </row>
     <row r="199" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11754,7 +11772,7 @@
         <v>353</v>
       </c>
       <c r="V199" s="2" t="s">
-        <v>519</v>
+        <v>510</v>
       </c>
     </row>
     <row r="200" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11806,7 +11824,7 @@
         <v>353</v>
       </c>
       <c r="V200" s="2" t="s">
-        <v>519</v>
+        <v>510</v>
       </c>
     </row>
     <row r="201" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11856,7 +11874,7 @@
         <v>356</v>
       </c>
       <c r="V201" s="2" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
     </row>
     <row r="202" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11906,7 +11924,7 @@
         <v>356</v>
       </c>
       <c r="V202" s="2" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
     </row>
     <row r="203" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -11956,7 +11974,7 @@
         <v>356</v>
       </c>
       <c r="V203" s="2" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
     </row>
     <row r="204" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12006,7 +12024,7 @@
         <v>356</v>
       </c>
       <c r="V204" s="2" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
     </row>
     <row r="205" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12056,7 +12074,7 @@
         <v>356</v>
       </c>
       <c r="V205" s="2" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
     </row>
     <row r="206" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12106,7 +12124,7 @@
         <v>356</v>
       </c>
       <c r="V206" s="2" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
     </row>
     <row r="207" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12158,7 +12176,7 @@
         <v>362</v>
       </c>
       <c r="V207" s="2" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
     </row>
     <row r="208" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12210,7 +12228,7 @@
         <v>362</v>
       </c>
       <c r="V208" s="2" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
     </row>
     <row r="209" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12262,7 +12280,7 @@
         <v>362</v>
       </c>
       <c r="V209" s="2" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
     </row>
     <row r="210" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12314,7 +12332,7 @@
         <v>362</v>
       </c>
       <c r="V210" s="2" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
     </row>
     <row r="211" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12366,7 +12384,7 @@
         <v>362</v>
       </c>
       <c r="V211" s="2" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
     </row>
     <row r="212" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12418,7 +12436,7 @@
         <v>362</v>
       </c>
       <c r="V212" s="2" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
     </row>
     <row r="213" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12464,7 +12482,7 @@
       <c r="T213" s="2"/>
       <c r="U213" s="2"/>
       <c r="V213" s="2" t="s">
-        <v>522</v>
+        <v>513</v>
       </c>
     </row>
     <row r="214" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12514,7 +12532,7 @@
         <v>372</v>
       </c>
       <c r="V214" s="2" t="s">
-        <v>523</v>
+        <v>514</v>
       </c>
     </row>
     <row r="215" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12562,7 +12580,7 @@
       <c r="T215" s="2"/>
       <c r="U215" s="2"/>
       <c r="V215" s="2" t="s">
-        <v>524</v>
+        <v>515</v>
       </c>
     </row>
     <row r="216" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12612,7 +12630,7 @@
       <c r="T216" s="2"/>
       <c r="U216" s="2"/>
       <c r="V216" s="2" t="s">
-        <v>524</v>
+        <v>515</v>
       </c>
     </row>
     <row r="217" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12626,14 +12644,14 @@
         <v>363</v>
       </c>
       <c r="D217" s="2" t="s">
-        <v>378</v>
+        <v>539</v>
       </c>
       <c r="E217" s="2" t="s">
         <v>365</v>
       </c>
       <c r="F217" s="2"/>
       <c r="G217" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H217" s="2">
         <v>12</v>
@@ -12655,10 +12673,10 @@
       </c>
       <c r="T217" s="2"/>
       <c r="U217" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="V217" s="2" t="s">
-        <v>525</v>
+        <v>516</v>
       </c>
     </row>
     <row r="218" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12672,14 +12690,14 @@
         <v>363</v>
       </c>
       <c r="D218" s="2" t="s">
-        <v>378</v>
+        <v>539</v>
       </c>
       <c r="E218" s="2" t="s">
         <v>376</v>
       </c>
       <c r="F218" s="2"/>
       <c r="G218" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="H218" s="2">
         <v>4</v>
@@ -12701,10 +12719,10 @@
       </c>
       <c r="T218" s="2"/>
       <c r="U218" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="V218" s="2" t="s">
-        <v>525</v>
+        <v>516</v>
       </c>
     </row>
     <row r="219" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12718,16 +12736,16 @@
         <v>363</v>
       </c>
       <c r="D219" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="E219" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="F219" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="G219" s="2" t="s">
         <v>378</v>
-      </c>
-      <c r="E219" s="2" t="s">
-        <v>382</v>
-      </c>
-      <c r="F219" s="2" t="s">
-        <v>383</v>
-      </c>
-      <c r="G219" s="2" t="s">
-        <v>379</v>
       </c>
       <c r="H219" s="2">
         <v>1</v>
@@ -12749,10 +12767,10 @@
       </c>
       <c r="T219" s="2"/>
       <c r="U219" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="V219" s="2" t="s">
-        <v>525</v>
+        <v>516</v>
       </c>
     </row>
     <row r="220" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12766,14 +12784,14 @@
         <v>363</v>
       </c>
       <c r="D220" s="2" t="s">
-        <v>378</v>
+        <v>539</v>
       </c>
       <c r="E220" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F220" s="2"/>
       <c r="G220" s="2" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="H220" s="2">
         <v>1</v>
@@ -12795,10 +12813,10 @@
       </c>
       <c r="T220" s="2"/>
       <c r="U220" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="V220" s="2" t="s">
-        <v>525</v>
+        <v>516</v>
       </c>
     </row>
     <row r="221" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12812,16 +12830,16 @@
         <v>363</v>
       </c>
       <c r="D221" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E221" s="2" t="s">
         <v>365</v>
       </c>
       <c r="F221" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="G221" s="2" t="s">
         <v>386</v>
-      </c>
-      <c r="G221" s="2" t="s">
-        <v>387</v>
       </c>
       <c r="H221" s="2">
         <v>12</v>
@@ -12835,7 +12853,7 @@
       <c r="M221" s="2"/>
       <c r="N221" s="2"/>
       <c r="O221" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="P221" s="2"/>
       <c r="Q221" s="2"/>
@@ -12846,7 +12864,7 @@
       <c r="T221" s="2"/>
       <c r="U221" s="2"/>
       <c r="V221" s="2" t="s">
-        <v>526</v>
+        <v>517</v>
       </c>
     </row>
     <row r="222" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12860,14 +12878,14 @@
         <v>363</v>
       </c>
       <c r="D222" s="2" t="s">
-        <v>389</v>
+        <v>540</v>
       </c>
       <c r="E222" s="2" t="s">
         <v>365</v>
       </c>
       <c r="F222" s="2"/>
       <c r="G222" s="2" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="H222" s="2">
         <v>12</v>
@@ -12889,10 +12907,10 @@
       </c>
       <c r="T222" s="2"/>
       <c r="U222" s="2" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="V222" s="2" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="223" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12906,16 +12924,16 @@
         <v>363</v>
       </c>
       <c r="D223" s="2" t="s">
-        <v>389</v>
+        <v>540</v>
       </c>
       <c r="E223" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F223" s="2" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="G223" s="2" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="H223" s="2">
         <v>1</v>
@@ -12937,10 +12955,10 @@
       </c>
       <c r="T223" s="2"/>
       <c r="U223" s="2" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="V223" s="2" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="224" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -12954,14 +12972,14 @@
         <v>363</v>
       </c>
       <c r="D224" s="2" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E224" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F224" s="2"/>
       <c r="G224" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="H224" s="2">
         <v>1</v>
@@ -12977,7 +12995,7 @@
       <c r="M224" s="2"/>
       <c r="N224" s="2"/>
       <c r="O224" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="P224" s="2"/>
       <c r="Q224" s="2"/>
@@ -12985,10 +13003,10 @@
       <c r="S224" s="2"/>
       <c r="T224" s="2"/>
       <c r="U224" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="V224" s="2" t="s">
-        <v>527</v>
+        <v>518</v>
       </c>
     </row>
     <row r="225" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13002,14 +13020,14 @@
         <v>363</v>
       </c>
       <c r="D225" s="2" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E225" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F225" s="2"/>
       <c r="G225" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="H225" s="2">
         <v>1</v>
@@ -13025,7 +13043,7 @@
       <c r="M225" s="2"/>
       <c r="N225" s="2"/>
       <c r="O225" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="P225" s="2"/>
       <c r="Q225" s="2"/>
@@ -13033,10 +13051,10 @@
       <c r="S225" s="2"/>
       <c r="T225" s="2"/>
       <c r="U225" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="V225" s="2" t="s">
-        <v>527</v>
+        <v>518</v>
       </c>
     </row>
     <row r="226" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13050,14 +13068,14 @@
         <v>363</v>
       </c>
       <c r="D226" s="2" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E226" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F226" s="2"/>
       <c r="G226" s="2" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="H226" s="2">
         <v>2</v>
@@ -13073,7 +13091,7 @@
       <c r="M226" s="2"/>
       <c r="N226" s="2"/>
       <c r="O226" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="P226" s="2"/>
       <c r="Q226" s="2"/>
@@ -13081,10 +13099,10 @@
       <c r="S226" s="2"/>
       <c r="T226" s="2"/>
       <c r="U226" s="2" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="V226" s="2" t="s">
-        <v>527</v>
+        <v>518</v>
       </c>
     </row>
     <row r="227" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13098,14 +13116,14 @@
         <v>363</v>
       </c>
       <c r="D227" s="2" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E227" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F227" s="2"/>
       <c r="G227" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="H227" s="2">
         <v>1</v>
@@ -13115,7 +13133,7 @@
       </c>
       <c r="J227" s="2"/>
       <c r="K227" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="L227" s="2"/>
       <c r="M227" s="2"/>
@@ -13127,10 +13145,10 @@
       <c r="S227" s="2"/>
       <c r="T227" s="2"/>
       <c r="U227" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="V227" s="2" t="s">
-        <v>528</v>
+        <v>519</v>
       </c>
     </row>
     <row r="228" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13144,14 +13162,14 @@
         <v>363</v>
       </c>
       <c r="D228" s="2" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E228" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F228" s="2"/>
       <c r="G228" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="H228" s="2">
         <v>1</v>
@@ -13161,7 +13179,7 @@
       </c>
       <c r="J228" s="2"/>
       <c r="K228" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="L228" s="2"/>
       <c r="M228" s="2"/>
@@ -13173,10 +13191,10 @@
       <c r="S228" s="2"/>
       <c r="T228" s="2"/>
       <c r="U228" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="V228" s="2" t="s">
-        <v>528</v>
+        <v>519</v>
       </c>
     </row>
     <row r="229" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13190,14 +13208,14 @@
         <v>363</v>
       </c>
       <c r="D229" s="2" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E229" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F229" s="2"/>
       <c r="G229" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="H229" s="2">
         <v>2</v>
@@ -13207,7 +13225,7 @@
       </c>
       <c r="J229" s="2"/>
       <c r="K229" s="2" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="L229" s="2"/>
       <c r="M229" s="2"/>
@@ -13219,10 +13237,10 @@
       <c r="S229" s="2"/>
       <c r="T229" s="2"/>
       <c r="U229" s="2" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="V229" s="2" t="s">
-        <v>528</v>
+        <v>519</v>
       </c>
     </row>
     <row r="230" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13236,16 +13254,16 @@
         <v>363</v>
       </c>
       <c r="D230" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E230" s="2" t="s">
         <v>365</v>
       </c>
       <c r="F230" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="G230" s="2" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="H230" s="2">
         <v>12</v>
@@ -13255,13 +13273,13 @@
       </c>
       <c r="J230" s="2"/>
       <c r="K230" s="2" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="L230" s="2"/>
       <c r="M230" s="2"/>
       <c r="N230" s="2"/>
       <c r="O230" s="2" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="P230" s="2"/>
       <c r="Q230" s="2"/>
@@ -13269,10 +13287,10 @@
       <c r="S230" s="2"/>
       <c r="T230" s="2"/>
       <c r="U230" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="V230" s="2" t="s">
-        <v>529</v>
+        <v>520</v>
       </c>
     </row>
     <row r="231" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13286,14 +13304,14 @@
         <v>363</v>
       </c>
       <c r="D231" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E231" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F231" s="2"/>
       <c r="G231" s="2" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="H231" s="2">
         <v>1</v>
@@ -13303,13 +13321,13 @@
       </c>
       <c r="J231" s="2"/>
       <c r="K231" s="2" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="L231" s="2"/>
       <c r="M231" s="2"/>
       <c r="N231" s="2"/>
       <c r="O231" s="2" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="P231" s="2"/>
       <c r="Q231" s="2"/>
@@ -13317,10 +13335,10 @@
       <c r="S231" s="2"/>
       <c r="T231" s="2"/>
       <c r="U231" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="V231" s="2" t="s">
-        <v>529</v>
+        <v>520</v>
       </c>
     </row>
     <row r="232" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13334,14 +13352,14 @@
         <v>363</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E232" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F232" s="2"/>
       <c r="G232" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="H232" s="2">
         <v>1</v>
@@ -13351,13 +13369,13 @@
       </c>
       <c r="J232" s="2"/>
       <c r="K232" s="2" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="L232" s="2"/>
       <c r="M232" s="2"/>
       <c r="N232" s="2"/>
       <c r="O232" s="2" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="P232" s="2"/>
       <c r="Q232" s="2"/>
@@ -13365,10 +13383,10 @@
       <c r="S232" s="2"/>
       <c r="T232" s="2"/>
       <c r="U232" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="V232" s="2" t="s">
-        <v>529</v>
+        <v>520</v>
       </c>
     </row>
     <row r="233" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13382,14 +13400,14 @@
         <v>363</v>
       </c>
       <c r="D233" s="2" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E233" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F233" s="2"/>
       <c r="G233" s="2" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="H233" s="2">
         <v>1</v>
@@ -13399,13 +13417,13 @@
       </c>
       <c r="J233" s="2"/>
       <c r="K233" s="2" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="L233" s="2"/>
       <c r="M233" s="2"/>
       <c r="N233" s="2"/>
       <c r="O233" s="2" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="P233" s="2"/>
       <c r="Q233" s="2"/>
@@ -13413,10 +13431,10 @@
       <c r="S233" s="2"/>
       <c r="T233" s="2"/>
       <c r="U233" s="2" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="V233" s="2" t="s">
-        <v>529</v>
+        <v>520</v>
       </c>
     </row>
     <row r="234" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13430,14 +13448,14 @@
         <v>363</v>
       </c>
       <c r="D234" s="2" t="s">
-        <v>409</v>
+        <v>541</v>
       </c>
       <c r="E234" s="2" t="s">
         <v>365</v>
       </c>
       <c r="F234" s="2"/>
       <c r="G234" s="2" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="H234" s="2">
         <v>12</v>
@@ -13457,10 +13475,10 @@
       <c r="S234" s="2"/>
       <c r="T234" s="2"/>
       <c r="U234" s="2" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="V234" s="2" t="s">
-        <v>530</v>
+        <v>521</v>
       </c>
     </row>
     <row r="235" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13474,16 +13492,16 @@
         <v>363</v>
       </c>
       <c r="D235" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="E235" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="E235" s="2" t="s">
-        <v>412</v>
-      </c>
       <c r="F235" s="2" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="G235" s="2" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="H235" s="2">
         <v>4</v>
@@ -13503,10 +13521,10 @@
       <c r="S235" s="2"/>
       <c r="T235" s="2"/>
       <c r="U235" s="2" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="V235" s="2" t="s">
-        <v>531</v>
+        <v>522</v>
       </c>
     </row>
     <row r="236" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13520,16 +13538,16 @@
         <v>363</v>
       </c>
       <c r="D236" s="2" t="s">
-        <v>409</v>
+        <v>541</v>
       </c>
       <c r="E236" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="F236" s="2" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="G236" s="2" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="H236" s="2">
         <v>1</v>
@@ -13549,10 +13567,10 @@
       <c r="S236" s="2"/>
       <c r="T236" s="2"/>
       <c r="U236" s="2" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="V236" s="2" t="s">
-        <v>531</v>
+        <v>522</v>
       </c>
     </row>
     <row r="237" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13566,16 +13584,16 @@
         <v>363</v>
       </c>
       <c r="D237" s="2" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E237" s="2" t="s">
         <v>365</v>
       </c>
       <c r="F237" s="2" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="G237" s="2" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="H237" s="2">
         <v>12</v>
@@ -13591,7 +13609,7 @@
       <c r="M237" s="2"/>
       <c r="N237" s="2"/>
       <c r="O237" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="P237" s="2"/>
       <c r="Q237" s="2"/>
@@ -13599,10 +13617,10 @@
       <c r="S237" s="2"/>
       <c r="T237" s="2"/>
       <c r="U237" s="2" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="V237" s="2" t="s">
-        <v>532</v>
+        <v>523</v>
       </c>
     </row>
     <row r="238" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13616,16 +13634,16 @@
         <v>363</v>
       </c>
       <c r="D238" s="2" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="E238" s="2" t="s">
         <v>365</v>
       </c>
       <c r="F238" s="2" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="G238" s="2" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="H238" s="2">
         <v>12</v>
@@ -13639,7 +13657,7 @@
       <c r="M238" s="2"/>
       <c r="N238" s="2"/>
       <c r="O238" s="2" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="P238" s="2"/>
       <c r="Q238" s="2"/>
@@ -13647,10 +13665,10 @@
       <c r="S238" s="2"/>
       <c r="T238" s="2"/>
       <c r="U238" s="2" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="V238" s="2" t="s">
-        <v>533</v>
+        <v>524</v>
       </c>
     </row>
     <row r="239" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13664,14 +13682,14 @@
         <v>363</v>
       </c>
       <c r="D239" s="2" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="E239" s="2" t="s">
         <v>365</v>
       </c>
       <c r="F239" s="2"/>
       <c r="G239" s="2" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="H239" s="2">
         <v>12</v>
@@ -13689,14 +13707,14 @@
       <c r="Q239" s="2"/>
       <c r="R239" s="2"/>
       <c r="S239" s="2" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="T239" s="2"/>
       <c r="U239" s="2" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="V239" s="2" t="s">
-        <v>534</v>
+        <v>525</v>
       </c>
     </row>
     <row r="240" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13710,14 +13728,14 @@
         <v>363</v>
       </c>
       <c r="D240" s="2" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="E240" s="2" t="s">
         <v>365</v>
       </c>
       <c r="F240" s="2"/>
       <c r="G240" s="2" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="H240" s="2">
         <v>12</v>
@@ -13727,7 +13745,7 @@
       </c>
       <c r="J240" s="2"/>
       <c r="K240" s="2" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="L240" s="2"/>
       <c r="M240" s="2"/>
@@ -13739,10 +13757,10 @@
       <c r="S240" s="2"/>
       <c r="T240" s="2"/>
       <c r="U240" s="2" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="V240" s="2" t="s">
-        <v>535</v>
+        <v>526</v>
       </c>
     </row>
     <row r="241" spans="1:22" s="15" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13756,16 +13774,16 @@
         <v>363</v>
       </c>
       <c r="D241" s="12" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E241" s="12" t="s">
         <v>365</v>
       </c>
       <c r="F241" s="12" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="G241" s="12" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="H241" s="12">
         <v>12</v>
@@ -13781,7 +13799,7 @@
       <c r="M241" s="12"/>
       <c r="N241" s="12"/>
       <c r="O241" s="12" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="P241" s="12"/>
       <c r="Q241" s="12"/>
@@ -13789,10 +13807,10 @@
       <c r="S241" s="12"/>
       <c r="T241" s="12"/>
       <c r="U241" s="12" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="V241" s="12" t="s">
-        <v>472</v>
+        <v>463</v>
       </c>
     </row>
     <row r="242" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13800,20 +13818,20 @@
         <v>22</v>
       </c>
       <c r="B242" s="8" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="C242" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D242" s="2" t="s">
-        <v>432</v>
+        <v>542</v>
       </c>
       <c r="E242" s="2" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="F242" s="2"/>
       <c r="G242" s="2" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="H242" s="2">
         <v>12</v>
@@ -13831,14 +13849,14 @@
       <c r="Q242" s="2"/>
       <c r="R242" s="2"/>
       <c r="S242" s="2" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
       <c r="T242" s="2"/>
       <c r="U242" s="2" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="V242" s="2" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
     </row>
     <row r="243" spans="1:22" s="15" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13846,20 +13864,20 @@
         <v>22</v>
       </c>
       <c r="B243" s="13" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
       <c r="C243" s="12" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D243" s="12" t="s">
-        <v>439</v>
+        <v>543</v>
       </c>
       <c r="E243" s="12" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="F243" s="12"/>
       <c r="G243" s="12" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="H243" s="12">
         <v>12</v>
@@ -13881,10 +13899,10 @@
       </c>
       <c r="T243" s="12"/>
       <c r="U243" s="12" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="V243" s="12" t="s">
-        <v>536</v>
+        <v>527</v>
       </c>
     </row>
     <row r="244" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13892,20 +13910,20 @@
         <v>22</v>
       </c>
       <c r="B244" s="8" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="C244" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D244" s="2" t="s">
-        <v>443</v>
+        <v>544</v>
       </c>
       <c r="E244" s="2" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="F244" s="2"/>
       <c r="G244" s="2" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="H244" s="2">
         <v>12</v>
@@ -13928,7 +13946,7 @@
       <c r="T244" s="2"/>
       <c r="U244" s="2"/>
       <c r="V244" s="2" t="s">
-        <v>469</v>
+        <v>460</v>
       </c>
     </row>
     <row r="245" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13939,17 +13957,17 @@
         <v>21647</v>
       </c>
       <c r="C245" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D245" s="2" t="s">
-        <v>445</v>
+        <v>536</v>
       </c>
       <c r="E245" s="2" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="F245" s="2"/>
       <c r="G245" s="2" t="s">
-        <v>446</v>
+        <v>439</v>
       </c>
       <c r="H245" s="2">
         <v>12</v>
@@ -13971,10 +13989,10 @@
       </c>
       <c r="T245" s="2"/>
       <c r="U245" s="2" t="s">
-        <v>473</v>
+        <v>464</v>
       </c>
       <c r="V245" s="2" t="s">
-        <v>471</v>
+        <v>462</v>
       </c>
     </row>
     <row r="246" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -13985,15 +14003,17 @@
         <v>21648</v>
       </c>
       <c r="C246" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="D246" s="2"/>
+        <v>428</v>
+      </c>
+      <c r="D246" s="2" t="s">
+        <v>538</v>
+      </c>
       <c r="E246" s="2" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="F246" s="2"/>
       <c r="G246" s="2" t="s">
-        <v>447</v>
+        <v>440</v>
       </c>
       <c r="H246" s="2">
         <v>12</v>
@@ -14016,7 +14036,7 @@
       <c r="T246" s="2"/>
       <c r="U246" s="2"/>
       <c r="V246" s="2" t="s">
-        <v>470</v>
+        <v>461</v>
       </c>
     </row>
     <row r="247" spans="1:22" s="15" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -14027,17 +14047,17 @@
         <v>24704</v>
       </c>
       <c r="C247" s="12" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D247" s="12" t="s">
-        <v>448</v>
+        <v>441</v>
       </c>
       <c r="E247" s="12" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="F247" s="12"/>
       <c r="G247" s="12" t="s">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="H247" s="12">
         <v>20</v>
@@ -14060,7 +14080,7 @@
       <c r="T247" s="12"/>
       <c r="U247" s="12"/>
       <c r="V247" s="12" t="s">
-        <v>537</v>
+        <v>528</v>
       </c>
     </row>
     <row r="248" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -14071,17 +14091,17 @@
         <v>46161</v>
       </c>
       <c r="C248" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D248" s="2" t="s">
-        <v>439</v>
+        <v>538</v>
       </c>
       <c r="E248" s="2" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
       <c r="F248" s="2"/>
       <c r="G248" s="2" t="s">
-        <v>450</v>
+        <v>443</v>
       </c>
       <c r="H248" s="2">
         <v>12</v>
@@ -14104,7 +14124,7 @@
       <c r="T248" s="2"/>
       <c r="U248" s="2"/>
       <c r="V248" s="2" t="s">
-        <v>538</v>
+        <v>529</v>
       </c>
     </row>
     <row r="249" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -14115,17 +14135,17 @@
         <v>101170</v>
       </c>
       <c r="C249" s="2" t="s">
-        <v>451</v>
+        <v>444</v>
       </c>
       <c r="D249" s="2" t="s">
-        <v>452</v>
+        <v>534</v>
       </c>
       <c r="E249" s="2" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="F249" s="2"/>
       <c r="G249" s="2" t="s">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="H249" s="2">
         <v>20</v>
@@ -14147,10 +14167,10 @@
       </c>
       <c r="T249" s="2"/>
       <c r="U249" s="2" t="s">
-        <v>455</v>
+        <v>447</v>
       </c>
       <c r="V249" s="2" t="s">
-        <v>539</v>
+        <v>530</v>
       </c>
     </row>
     <row r="250" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -14161,17 +14181,17 @@
         <v>101171</v>
       </c>
       <c r="C250" s="2" t="s">
-        <v>451</v>
+        <v>444</v>
       </c>
       <c r="D250" s="2" t="s">
-        <v>452</v>
+        <v>534</v>
       </c>
       <c r="E250" s="2" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="F250" s="2"/>
       <c r="G250" s="2" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
       <c r="H250" s="2">
         <v>12</v>
@@ -14193,10 +14213,10 @@
       </c>
       <c r="T250" s="2"/>
       <c r="U250" s="2" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="V250" s="2" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
     </row>
     <row r="251" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -14207,17 +14227,17 @@
         <v>101172</v>
       </c>
       <c r="C251" s="2" t="s">
-        <v>451</v>
+        <v>444</v>
       </c>
       <c r="D251" s="2" t="s">
-        <v>452</v>
+        <v>534</v>
       </c>
       <c r="E251" s="2" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="F251" s="2"/>
       <c r="G251" s="2" t="s">
-        <v>459</v>
+        <v>451</v>
       </c>
       <c r="H251" s="2">
         <v>12</v>
@@ -14239,10 +14259,10 @@
       </c>
       <c r="T251" s="2"/>
       <c r="U251" s="2" t="s">
-        <v>460</v>
+        <v>452</v>
       </c>
       <c r="V251" s="2" t="s">
-        <v>540</v>
+        <v>531</v>
       </c>
     </row>
     <row r="252" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -14250,18 +14270,20 @@
         <v>22</v>
       </c>
       <c r="B252" s="8" t="s">
-        <v>461</v>
+        <v>453</v>
       </c>
       <c r="C252" s="2" t="s">
-        <v>462</v>
-      </c>
-      <c r="D252" s="2"/>
+        <v>454</v>
+      </c>
+      <c r="D252" s="2" t="s">
+        <v>536</v>
+      </c>
       <c r="E252" s="2" t="s">
-        <v>463</v>
+        <v>455</v>
       </c>
       <c r="F252" s="2"/>
       <c r="G252" s="2" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
       <c r="H252" s="2">
         <v>20</v>
@@ -14284,28 +14306,28 @@
       <c r="T252" s="2"/>
       <c r="U252" s="2"/>
       <c r="V252" s="2" t="s">
-        <v>541</v>
+        <v>532</v>
       </c>
     </row>
     <row r="253" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A253" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B253" s="8">
+      <c r="A253" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B253" s="13">
         <v>170367</v>
       </c>
       <c r="C253" s="2" t="s">
-        <v>465</v>
+        <v>457</v>
       </c>
       <c r="D253" s="2" t="s">
-        <v>466</v>
+        <v>535</v>
       </c>
       <c r="E253" s="2" t="s">
         <v>365</v>
       </c>
       <c r="F253" s="2"/>
       <c r="G253" s="2" t="s">
-        <v>467</v>
+        <v>458</v>
       </c>
       <c r="H253" s="2">
         <v>12</v>
@@ -14325,31 +14347,90 @@
       <c r="S253" s="2"/>
       <c r="T253" s="2"/>
       <c r="U253" s="2" t="s">
-        <v>468</v>
+        <v>459</v>
       </c>
       <c r="V253" s="2" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="254" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="255" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="256" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="257" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="258" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="259" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="260" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="261" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="262" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="263" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="264" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="265" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="266" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="267" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="268" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="269" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="270" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="271" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="272" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>533</v>
+      </c>
+    </row>
+    <row r="254" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A254" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B254" s="16" t="s">
+        <v>537</v>
+      </c>
+      <c r="C254" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="D254" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="E254" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="F254" s="2"/>
+      <c r="G254" s="2" t="s">
+        <v>456</v>
+      </c>
+      <c r="I254" s="11">
+        <v>60</v>
+      </c>
+      <c r="S254" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V254" s="2" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="255" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A255" s="12"/>
+      <c r="B255" s="16"/>
+    </row>
+    <row r="256" spans="1:22" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A256" s="12"/>
+      <c r="B256" s="16"/>
+    </row>
+    <row r="257" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A257" s="12"/>
+      <c r="B257" s="16"/>
+    </row>
+    <row r="258" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A258" s="15"/>
+      <c r="B258" s="16"/>
+    </row>
+    <row r="259" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A259" s="15"/>
+      <c r="B259" s="16"/>
+    </row>
+    <row r="260" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A260" s="15"/>
+      <c r="B260" s="16"/>
+    </row>
+    <row r="261" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A261" s="15"/>
+      <c r="B261" s="16"/>
+    </row>
+    <row r="262" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A262" s="15"/>
+      <c r="B262" s="16"/>
+    </row>
+    <row r="263" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A263" s="15"/>
+      <c r="B263" s="16"/>
+    </row>
+    <row r="264" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A264" s="15"/>
+      <c r="B264" s="16"/>
+    </row>
+    <row r="265" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="266" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="267" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="268" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="269" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="270" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="271" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="272" spans="1:2" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="273" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="274" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="275" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -15113,6 +15194,9 @@
     <row r="1033" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A1:V253" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="B1:B1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>

</xml_diff>